<commit_message>
KPI actualizado 2026-08-27 19:08 UTC
</commit_message>
<xml_diff>
--- a/data/50001449 -  Itaberaba Extracción.xlsx
+++ b/data/50001449 -  Itaberaba Extracción.xlsx
@@ -173,25 +173,25 @@
     <t>Propuesta Motor  OT4080</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
+    <t>1217786049371846</t>
+  </si>
+  <si>
+    <t>Ingenieria Nucleo Rodete  OT4080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación oc Alabes OT4080,Propuesta nucleo Rodete  OT4080 </t>
+  </si>
+  <si>
+    <t>1217786388836063</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Plano Preliminar  OT4080</t>
+  </si>
+  <si>
     <t>Baja</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1217786049371846</t>
-  </si>
-  <si>
-    <t>Ingenieria Nucleo Rodete  OT4080</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación oc Alabes OT4080,Propuesta nucleo Rodete  OT4080 </t>
-  </si>
-  <si>
-    <t>1217786388836063</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Plano Preliminar  OT4080</t>
   </si>
   <si>
     <t>1217783436184652</t>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="9">
-        <v>46260.17370655092</v>
+        <v>46261.20674524306</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>43</v>
@@ -1884,29 +1884,29 @@
       <c r="R9" s="9">
         <v>46259</v>
       </c>
-      <c r="S9" s="7" t="s">
-        <v>45</v>
+      <c r="S9" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T9" s="10">
         <v>0</v>
       </c>
       <c r="U9" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="5">
         <v>46258.603081203706</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46260.1737024537</v>
+        <v>46261.2067450926</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>26</v>
@@ -1939,7 +1939,7 @@
         <v>37</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q10" s="5">
         <v>46260</v>
@@ -1947,19 +1947,19 @@
       <c r="R10" s="5">
         <v>46259</v>
       </c>
-      <c r="S10" s="7" t="s">
-        <v>45</v>
+      <c r="S10" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T10" s="6">
         <v>0</v>
       </c>
       <c r="U10" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="9">
         <v>46258.60308479167</v>
@@ -2002,7 +2002,7 @@
         <v>37</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Q11" s="9">
         <v>46262</v>
@@ -2011,13 +2011,13 @@
         <v>46259</v>
       </c>
       <c r="S11" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T11" s="10">
         <v>0</v>
       </c>
       <c r="U11" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -2121,7 +2121,7 @@
         <v>46325</v>
       </c>
       <c r="S13" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T13" s="10">
         <v>0</v>
@@ -2184,7 +2184,7 @@
         <v>46325</v>
       </c>
       <c r="S14" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T14" s="6">
         <v>0</v>
@@ -2247,7 +2247,7 @@
         <v>46325</v>
       </c>
       <c r="S15" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T15" s="10">
         <v>0</v>
@@ -2310,7 +2310,7 @@
         <v>46325</v>
       </c>
       <c r="S16" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T16" s="6">
         <v>0</v>
@@ -2373,7 +2373,7 @@
         <v>46261</v>
       </c>
       <c r="S17" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T17" s="10">
         <v>0</v>
@@ -2424,7 +2424,7 @@
         <v>53</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>74</v>
@@ -2436,7 +2436,7 @@
         <v>46261</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T18" s="6">
         <v>0</v>
@@ -2546,7 +2546,7 @@
         <v>46329</v>
       </c>
       <c r="S20" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T20" s="6">
         <v>0</v>
@@ -2715,7 +2715,7 @@
         <v>46329</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T23" s="10">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>46329</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T26" s="6">
         <v>0</v>
@@ -3053,7 +3053,7 @@
         <v>46329</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T29" s="10">
         <v>0</v>
@@ -3275,7 +3275,7 @@
         <v>46265</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T33" s="10">
         <v>0</v>
@@ -3497,7 +3497,7 @@
         <v>46261</v>
       </c>
       <c r="S37" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T37" s="10">
         <v>0</v>
@@ -3548,7 +3548,7 @@
         <v>132</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>136</v>
@@ -3713,7 +3713,7 @@
         <v>46265</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T41" s="10">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         <v>46304</v>
       </c>
       <c r="S42" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T42" s="6">
         <v>0</v>
@@ -3839,7 +3839,7 @@
         <v>46324</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T43" s="10">
         <v>0</v>
@@ -3902,7 +3902,7 @@
         <v>46429</v>
       </c>
       <c r="S44" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T44" s="6">
         <v>0</v>
@@ -4118,7 +4118,7 @@
         <v>46340</v>
       </c>
       <c r="S48" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T48" s="6">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         <v>46343</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T49" s="10">
         <v>0</v>
@@ -4244,7 +4244,7 @@
         <v>46340</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
@@ -4307,7 +4307,7 @@
         <v>46343</v>
       </c>
       <c r="S51" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T51" s="10">
         <v>0</v>
@@ -4370,7 +4370,7 @@
         <v>46340</v>
       </c>
       <c r="S52" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T52" s="6">
         <v>0</v>
@@ -4433,7 +4433,7 @@
         <v>46343</v>
       </c>
       <c r="S53" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T53" s="10">
         <v>0</v>
@@ -4543,7 +4543,7 @@
         <v>46345</v>
       </c>
       <c r="S55" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T55" s="10">
         <v>0</v>
@@ -4606,7 +4606,7 @@
         <v>46365</v>
       </c>
       <c r="S56" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T56" s="6">
         <v>0</v>
@@ -4775,7 +4775,7 @@
         <v>46394</v>
       </c>
       <c r="S59" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T59" s="10">
         <v>0</v>
@@ -4991,7 +4991,7 @@
         <v>46349</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T63" s="10">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>46386</v>
       </c>
       <c r="S64" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T64" s="6">
         <v>0</v>
@@ -5164,7 +5164,7 @@
         <v>46395</v>
       </c>
       <c r="S66" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T66" s="6">
         <v>0</v>
@@ -5333,7 +5333,7 @@
         <v>46415</v>
       </c>
       <c r="S69" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T69" s="10">
         <v>0</v>
@@ -5502,7 +5502,7 @@
         <v>46419</v>
       </c>
       <c r="S72" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T72" s="6">
         <v>0</v>
@@ -5671,7 +5671,7 @@
         <v>46421</v>
       </c>
       <c r="S75" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T75" s="10">
         <v>0</v>
@@ -5840,7 +5840,7 @@
         <v>46423</v>
       </c>
       <c r="S78" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T78" s="6">
         <v>0</v>
@@ -6009,7 +6009,7 @@
         <v>46427</v>
       </c>
       <c r="S81" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T81" s="10">
         <v>0</v>
@@ -6178,7 +6178,7 @@
         <v>46433</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
@@ -6394,7 +6394,7 @@
         <v>46435</v>
       </c>
       <c r="S88" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T88" s="6">
         <v>0</v>
@@ -6563,7 +6563,7 @@
         <v>46437</v>
       </c>
       <c r="S91" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T91" s="10">
         <v>0</v>
@@ -6732,7 +6732,7 @@
         <v>46441</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
@@ -6901,7 +6901,7 @@
         <v>46443</v>
       </c>
       <c r="S97" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T97" s="10">
         <v>0</v>
@@ -7117,7 +7117,7 @@
         <v>46447</v>
       </c>
       <c r="S101" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T101" s="10">
         <v>0</v>
@@ -7180,7 +7180,7 @@
         <v>46447</v>
       </c>
       <c r="S102" s="7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="T102" s="6">
         <v>0</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-28 04:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001449 -  Itaberaba Extracción.xlsx
+++ b/data/50001449 -  Itaberaba Extracción.xlsx
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="9">
-        <v>46258.66330583333</v>
+        <v>46262.17503763889</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>41</v>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46258.65866444445</v>
+        <v>46262.175033067135</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>44</v>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46258.65865997685</v>
+        <v>46262.17503131945</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>73</v>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46258.65938915509</v>
+        <v>46262.175003275464</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-29 13:13 Chile
</commit_message>
<xml_diff>
--- a/data/50001449 -  Itaberaba Extracción.xlsx
+++ b/data/50001449 -  Itaberaba Extracción.xlsx
@@ -191,31 +191,31 @@
     <t>Ingenieria Jefe de proyecto:,Plano Preliminar  OT4080</t>
   </si>
   <si>
+    <t>1217783436184652</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta Corte laser  OT4080</t>
+  </si>
+  <si>
+    <t>1217786388836378</t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Check Planos  OT4080</t>
+  </si>
+  <si>
+    <t>Generacion OC Corte Laser  OT4080,Propuesta compras:</t>
+  </si>
+  <si>
     <t>Baja</t>
-  </si>
-  <si>
-    <t>1217783436184652</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta Corte laser  OT4080</t>
-  </si>
-  <si>
-    <t>1217786388836378</t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Check Planos  OT4080</t>
-  </si>
-  <si>
-    <t>Generacion OC Corte Laser  OT4080,Propuesta compras:</t>
   </si>
   <si>
     <t>Tarea sin iniciar</t>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="9">
-        <v>46262.17503763889</v>
+        <v>46263.20694251158</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>41</v>
@@ -2010,8 +2010,8 @@
       <c r="R11" s="9">
         <v>46259</v>
       </c>
-      <c r="S11" s="7" t="s">
-        <v>51</v>
+      <c r="S11" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T11" s="10">
         <v>0</v>
@@ -2022,7 +2022,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" s="5">
         <v>46258.60300328703</v>
@@ -2032,7 +2032,7 @@
         <v>46258.62771878472</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>25</v>
@@ -2056,7 +2056,7 @@
         <v>26</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P12" s="6" t="s">
         <v>26</v>
@@ -2069,7 +2069,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="9">
         <v>46258.603095555554</v>
@@ -2079,16 +2079,16 @@
         <v>46258.65862203704</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I13" s="9">
         <v>46325</v>
@@ -2106,13 +2106,13 @@
         <v>26</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O13" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="P13" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>59</v>
       </c>
       <c r="Q13" s="9">
         <v>46328</v>
@@ -2121,7 +2121,7 @@
         <v>46325</v>
       </c>
       <c r="S13" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T13" s="10">
         <v>0</v>
@@ -2148,10 +2148,10 @@
         <v>26</v>
       </c>
       <c r="G14" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I14" s="5">
         <v>46325</v>
@@ -2169,10 +2169,10 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>63</v>
@@ -2184,7 +2184,7 @@
         <v>46325</v>
       </c>
       <c r="S14" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T14" s="6">
         <v>0</v>
@@ -2211,10 +2211,10 @@
         <v>26</v>
       </c>
       <c r="G15" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I15" s="9">
         <v>46325</v>
@@ -2232,10 +2232,10 @@
         <v>26</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>66</v>
@@ -2247,7 +2247,7 @@
         <v>46325</v>
       </c>
       <c r="S15" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T15" s="10">
         <v>0</v>
@@ -2274,10 +2274,10 @@
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I16" s="5">
         <v>46325</v>
@@ -2295,10 +2295,10 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="P16" s="6" t="s">
         <v>69</v>
@@ -2310,7 +2310,7 @@
         <v>46325</v>
       </c>
       <c r="S16" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T16" s="6">
         <v>0</v>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46262.175033067135</v>
+        <v>46263.206942986115</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>44</v>
@@ -2358,7 +2358,7 @@
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>43</v>
@@ -2372,8 +2372,8 @@
       <c r="R17" s="9">
         <v>46261</v>
       </c>
-      <c r="S17" s="7" t="s">
-        <v>51</v>
+      <c r="S17" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T17" s="10">
         <v>0</v>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46262.17503131945</v>
+        <v>46263.20694233796</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>73</v>
@@ -2421,7 +2421,7 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>47</v>
@@ -2435,8 +2435,8 @@
       <c r="R18" s="5">
         <v>46261</v>
       </c>
-      <c r="S18" s="7" t="s">
-        <v>51</v>
+      <c r="S18" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T18" s="6">
         <v>0</v>
@@ -2546,7 +2546,7 @@
         <v>46329</v>
       </c>
       <c r="S20" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T20" s="6">
         <v>0</v>
@@ -2597,7 +2597,7 @@
         <v>77</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>84</v>
@@ -2715,7 +2715,7 @@
         <v>46329</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T23" s="10">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>46329</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T26" s="6">
         <v>0</v>
@@ -3053,7 +3053,7 @@
         <v>46329</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T29" s="10">
         <v>0</v>
@@ -3275,7 +3275,7 @@
         <v>46265</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T33" s="10">
         <v>0</v>
@@ -3497,7 +3497,7 @@
         <v>46261</v>
       </c>
       <c r="S37" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T37" s="10">
         <v>0</v>
@@ -3713,7 +3713,7 @@
         <v>46265</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T41" s="10">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         <v>46304</v>
       </c>
       <c r="S42" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T42" s="6">
         <v>0</v>
@@ -3797,7 +3797,7 @@
         <v>46258.65948893518</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
@@ -3839,7 +3839,7 @@
         <v>46324</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T43" s="10">
         <v>0</v>
@@ -3902,7 +3902,7 @@
         <v>46429</v>
       </c>
       <c r="S44" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T44" s="6">
         <v>0</v>
@@ -4118,7 +4118,7 @@
         <v>46340</v>
       </c>
       <c r="S48" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T48" s="6">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         <v>46343</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T49" s="10">
         <v>0</v>
@@ -4244,7 +4244,7 @@
         <v>46340</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
@@ -4307,7 +4307,7 @@
         <v>46343</v>
       </c>
       <c r="S51" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T51" s="10">
         <v>0</v>
@@ -4370,7 +4370,7 @@
         <v>46340</v>
       </c>
       <c r="S52" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T52" s="6">
         <v>0</v>
@@ -4433,7 +4433,7 @@
         <v>46343</v>
       </c>
       <c r="S53" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T53" s="10">
         <v>0</v>
@@ -4543,7 +4543,7 @@
         <v>46345</v>
       </c>
       <c r="S55" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T55" s="10">
         <v>0</v>
@@ -4606,7 +4606,7 @@
         <v>46365</v>
       </c>
       <c r="S56" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T56" s="6">
         <v>0</v>
@@ -4775,7 +4775,7 @@
         <v>46394</v>
       </c>
       <c r="S59" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T59" s="10">
         <v>0</v>
@@ -4991,7 +4991,7 @@
         <v>46349</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T63" s="10">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>46386</v>
       </c>
       <c r="S64" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T64" s="6">
         <v>0</v>
@@ -5128,10 +5128,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I66" s="5">
         <v>46395</v>
@@ -5164,7 +5164,7 @@
         <v>46395</v>
       </c>
       <c r="S66" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T66" s="6">
         <v>0</v>
@@ -5191,10 +5191,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I67" s="9">
         <v>46395</v>
@@ -5244,10 +5244,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I68" s="5">
         <v>46395</v>
@@ -5297,10 +5297,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I69" s="9">
         <v>46415</v>
@@ -5333,7 +5333,7 @@
         <v>46415</v>
       </c>
       <c r="S69" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T69" s="10">
         <v>0</v>
@@ -5360,10 +5360,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I70" s="5">
         <v>46415</v>
@@ -5413,10 +5413,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I71" s="9">
         <v>46415</v>
@@ -5466,10 +5466,10 @@
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I72" s="5">
         <v>46419</v>
@@ -5502,7 +5502,7 @@
         <v>46419</v>
       </c>
       <c r="S72" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T72" s="6">
         <v>0</v>
@@ -5529,10 +5529,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I73" s="9">
         <v>46419</v>
@@ -5582,10 +5582,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I74" s="5">
         <v>46419</v>
@@ -5635,10 +5635,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I75" s="9">
         <v>46421</v>
@@ -5671,7 +5671,7 @@
         <v>46421</v>
       </c>
       <c r="S75" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T75" s="10">
         <v>0</v>
@@ -5698,10 +5698,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I76" s="5">
         <v>46421</v>
@@ -5751,10 +5751,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I77" s="9">
         <v>46421</v>
@@ -5804,10 +5804,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I78" s="5">
         <v>46423</v>
@@ -5840,7 +5840,7 @@
         <v>46423</v>
       </c>
       <c r="S78" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T78" s="6">
         <v>0</v>
@@ -5867,10 +5867,10 @@
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H79" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I79" s="9">
         <v>46423</v>
@@ -5920,10 +5920,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I80" s="5">
         <v>46423</v>
@@ -5973,10 +5973,10 @@
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H81" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H81" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I81" s="9">
         <v>46427</v>
@@ -6009,7 +6009,7 @@
         <v>46427</v>
       </c>
       <c r="S81" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T81" s="10">
         <v>0</v>
@@ -6036,10 +6036,10 @@
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I82" s="5">
         <v>46427</v>
@@ -6089,10 +6089,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H83" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H83" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I83" s="9">
         <v>46427</v>
@@ -6142,10 +6142,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H84" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I84" s="5">
         <v>46433</v>
@@ -6178,7 +6178,7 @@
         <v>46433</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
@@ -6205,10 +6205,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H85" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H85" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I85" s="9">
         <v>46433</v>
@@ -6258,10 +6258,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I86" s="5">
         <v>46433</v>
@@ -6394,7 +6394,7 @@
         <v>46435</v>
       </c>
       <c r="S88" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T88" s="6">
         <v>0</v>
@@ -6527,10 +6527,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H91" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H91" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I91" s="9">
         <v>46437</v>
@@ -6563,7 +6563,7 @@
         <v>46437</v>
       </c>
       <c r="S91" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T91" s="10">
         <v>0</v>
@@ -6590,10 +6590,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H92" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="H92" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="I92" s="5">
         <v>46437</v>
@@ -6643,10 +6643,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H93" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="H93" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="I93" s="9">
         <v>46437</v>
@@ -6732,7 +6732,7 @@
         <v>46441</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
@@ -6901,7 +6901,7 @@
         <v>46443</v>
       </c>
       <c r="S97" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T97" s="10">
         <v>0</v>
@@ -7117,7 +7117,7 @@
         <v>46447</v>
       </c>
       <c r="S101" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T101" s="10">
         <v>0</v>
@@ -7180,7 +7180,7 @@
         <v>46447</v>
       </c>
       <c r="S102" s="7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="T102" s="6">
         <v>0</v>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-10 17:03 UTC
</commit_message>
<xml_diff>
--- a/data/50001449 -  Itaberaba Extracción.xlsx
+++ b/data/50001449 -  Itaberaba Extracción.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="296">
   <si>
     <t>50001449 - Itaberaba Extracción</t>
   </si>
@@ -480,6 +480,9 @@
   </si>
   <si>
     <t>Ingenieria y diseño:,Plano Definitivos  OT4080</t>
+  </si>
+  <si>
+    <t>Media</t>
   </si>
   <si>
     <t>1217786389021681</t>
@@ -3668,7 +3671,7 @@
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46258.659496168984</v>
+        <v>46275.141257511576</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>144</v>
@@ -3712,8 +3715,8 @@
       <c r="R41" s="9">
         <v>46265</v>
       </c>
-      <c r="S41" s="7" t="s">
-        <v>59</v>
+      <c r="S41" s="12" t="s">
+        <v>148</v>
       </c>
       <c r="T41" s="10">
         <v>0</v>
@@ -3724,7 +3727,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B42" s="5">
         <v>46258.60324565972</v>
@@ -3734,7 +3737,7 @@
         <v>46258.65949248843</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
@@ -3767,7 +3770,7 @@
         <v>144</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="Q42" s="5">
         <v>46323</v>
@@ -3787,7 +3790,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B43" s="9">
         <v>46258.603256365735</v>
@@ -3827,10 +3830,10 @@
         <v>141</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P43" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q43" s="9">
         <v>46324</v>
@@ -3850,7 +3853,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B44" s="5">
         <v>46258.603271354164</v>
@@ -3860,16 +3863,16 @@
         <v>46258.65958741898</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I44" s="5">
         <v>46429</v>
@@ -3890,10 +3893,10 @@
         <v>141</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q44" s="5">
         <v>46430</v>
@@ -3913,7 +3916,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B45" s="9">
         <v>46258.603279849536</v>
@@ -3923,16 +3926,16 @@
         <v>46258.65955380787</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I45" s="9">
         <v>46429</v>
@@ -3950,13 +3953,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -3966,7 +3969,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B46" s="5">
         <v>46258.603283703706</v>
@@ -3976,16 +3979,16 @@
         <v>46258.659549930555</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I46" s="5">
         <v>46429</v>
@@ -4003,13 +4006,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Q46" s="6"/>
       <c r="R46" s="6"/>
@@ -4019,7 +4022,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B47" s="9">
         <v>46258.60332472222</v>
@@ -4029,7 +4032,7 @@
         <v>46258.6397684838</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>25</v>
@@ -4053,7 +4056,7 @@
         <v>26</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P47" s="10" t="s">
         <v>26</v>
@@ -4066,7 +4069,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B48" s="5">
         <v>46258.603327777775</v>
@@ -4076,16 +4079,16 @@
         <v>46258.6596800463</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I48" s="5">
         <v>46340</v>
@@ -4103,13 +4106,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>86</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="Q48" s="5">
         <v>46342</v>
@@ -4129,7 +4132,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B49" s="9">
         <v>46258.603332569444</v>
@@ -4139,16 +4142,16 @@
         <v>46258.659676400464</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I49" s="9">
         <v>46343</v>
@@ -4166,13 +4169,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O49" s="10" t="s">
         <v>94</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Q49" s="9">
         <v>46344</v>
@@ -4192,7 +4195,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B50" s="5">
         <v>46258.603337152774</v>
@@ -4202,16 +4205,16 @@
         <v>46258.6596725</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I50" s="5">
         <v>46340</v>
@@ -4229,13 +4232,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>101</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q50" s="5">
         <v>46342</v>
@@ -4255,7 +4258,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B51" s="9">
         <v>46258.60334170139</v>
@@ -4265,7 +4268,7 @@
         <v>46258.65976054398</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
@@ -4292,13 +4295,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q51" s="9">
         <v>46344</v>
@@ -4318,7 +4321,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B52" s="5">
         <v>46258.6033465625</v>
@@ -4328,7 +4331,7 @@
         <v>46258.659756863424</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
@@ -4355,13 +4358,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q52" s="5">
         <v>46342</v>
@@ -4381,7 +4384,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B53" s="9">
         <v>46258.603351550926</v>
@@ -4391,7 +4394,7 @@
         <v>46258.65975280093</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>26</v>
@@ -4418,13 +4421,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="Q53" s="9">
         <v>46344</v>
@@ -4444,7 +4447,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B54" s="5">
         <v>46258.60335619213</v>
@@ -4454,7 +4457,7 @@
         <v>46258.6432152662</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>25</v>
@@ -4478,7 +4481,7 @@
         <v>26</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>26</v>
@@ -4491,7 +4494,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B55" s="9">
         <v>46258.60335866898</v>
@@ -4501,16 +4504,16 @@
         <v>46258.66044761574</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I55" s="9">
         <v>46345</v>
@@ -4528,13 +4531,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O55" s="10" t="s">
         <v>65</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q55" s="9">
         <v>46364</v>
@@ -4554,7 +4557,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B56" s="5">
         <v>46258.60336445602</v>
@@ -4564,16 +4567,16 @@
         <v>46258.66056923611</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I56" s="5">
         <v>46365</v>
@@ -4591,13 +4594,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="Q56" s="5">
         <v>46393</v>
@@ -4617,7 +4620,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B57" s="9">
         <v>46258.603369317134</v>
@@ -4627,16 +4630,16 @@
         <v>46258.660526875</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I57" s="9">
         <v>46365</v>
@@ -4654,13 +4657,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Q57" s="10"/>
       <c r="R57" s="10"/>
@@ -4670,7 +4673,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B58" s="5">
         <v>46258.603375694445</v>
@@ -4680,16 +4683,16 @@
         <v>46258.660523252314</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I58" s="5">
         <v>46365</v>
@@ -4707,13 +4710,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Q58" s="6"/>
       <c r="R58" s="6"/>
@@ -4723,7 +4726,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B59" s="9">
         <v>46258.603471724535</v>
@@ -4733,7 +4736,7 @@
         <v>46258.66070581018</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
@@ -4760,13 +4763,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="Q59" s="9">
         <v>46394</v>
@@ -4786,7 +4789,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B60" s="5">
         <v>46258.60347714121</v>
@@ -4796,7 +4799,7 @@
         <v>46258.66066758102</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
@@ -4823,13 +4826,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
@@ -4839,7 +4842,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B61" s="9">
         <v>46258.60348181713</v>
@@ -4849,7 +4852,7 @@
         <v>46258.660663946765</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
@@ -4876,13 +4879,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q61" s="10"/>
       <c r="R61" s="10"/>
@@ -4892,7 +4895,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B62" s="5">
         <v>46258.603526377316</v>
@@ -4902,7 +4905,7 @@
         <v>46258.64433164352</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>25</v>
@@ -4926,7 +4929,7 @@
         <v>26</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>26</v>
@@ -4939,7 +4942,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B63" s="9">
         <v>46258.60352935185</v>
@@ -4949,16 +4952,16 @@
         <v>46258.66076600694</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I63" s="9">
         <v>46349</v>
@@ -4976,13 +4979,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="O63" s="10" t="s">
         <v>138</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="Q63" s="9">
         <v>46349</v>
@@ -5002,7 +5005,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B64" s="5">
         <v>46258.60354351852</v>
@@ -5012,16 +5015,16 @@
         <v>46258.66076209491</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I64" s="5">
         <v>46386</v>
@@ -5039,13 +5042,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>127</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Q64" s="5">
         <v>46386</v>
@@ -5065,7 +5068,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B65" s="9">
         <v>46258.60355135417</v>
@@ -5075,7 +5078,7 @@
         <v>46258.64755980324</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>25</v>
@@ -5099,7 +5102,7 @@
         <v>26</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P65" s="10" t="s">
         <v>26</v>
@@ -5112,7 +5115,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B66" s="5">
         <v>46258.60355402778</v>
@@ -5122,7 +5125,7 @@
         <v>46258.66087590277</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5149,13 +5152,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Q66" s="5">
         <v>46414</v>
@@ -5175,7 +5178,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B67" s="9">
         <v>46258.6035587963</v>
@@ -5185,7 +5188,7 @@
         <v>46258.66092363426</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
@@ -5212,13 +5215,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Q67" s="10"/>
       <c r="R67" s="10"/>
@@ -5228,7 +5231,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B68" s="5">
         <v>46258.60356253472</v>
@@ -5238,7 +5241,7 @@
         <v>46258.66091918982</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5265,13 +5268,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Q68" s="6"/>
       <c r="R68" s="6"/>
@@ -5281,7 +5284,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B69" s="9">
         <v>46258.603590555555</v>
@@ -5291,7 +5294,7 @@
         <v>46258.660871782406</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
@@ -5318,13 +5321,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Q69" s="9">
         <v>46416</v>
@@ -5344,7 +5347,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B70" s="5">
         <v>46258.60359733796</v>
@@ -5354,7 +5357,7 @@
         <v>46258.66098734953</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5381,13 +5384,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5397,7 +5400,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B71" s="9">
         <v>46258.60360181713</v>
@@ -5407,7 +5410,7 @@
         <v>46258.66098335648</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
@@ -5434,13 +5437,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q71" s="10"/>
       <c r="R71" s="10"/>
@@ -5450,7 +5453,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B72" s="5">
         <v>46258.60369793982</v>
@@ -5460,7 +5463,7 @@
         <v>46258.660867824074</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
@@ -5487,13 +5490,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Q72" s="5">
         <v>46420</v>
@@ -5513,7 +5516,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B73" s="9">
         <v>46258.60370306713</v>
@@ -5523,7 +5526,7 @@
         <v>46258.66106049769</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
@@ -5550,13 +5553,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="Q73" s="10"/>
       <c r="R73" s="10"/>
@@ -5566,7 +5569,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B74" s="5">
         <v>46258.6037081713</v>
@@ -5576,7 +5579,7 @@
         <v>46258.6610559375</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5603,13 +5606,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
@@ -5619,7 +5622,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B75" s="9">
         <v>46258.60373736111</v>
@@ -5629,7 +5632,7 @@
         <v>46258.66086319444</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>26</v>
@@ -5656,13 +5659,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q75" s="9">
         <v>46422</v>
@@ -5682,7 +5685,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B76" s="5">
         <v>46258.603744305554</v>
@@ -5692,7 +5695,7 @@
         <v>46258.66111847222</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
@@ -5719,13 +5722,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -5735,7 +5738,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B77" s="9">
         <v>46258.603748368056</v>
@@ -5745,7 +5748,7 @@
         <v>46258.66111508102</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
@@ -5772,13 +5775,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="Q77" s="10"/>
       <c r="R77" s="10"/>
@@ -5788,7 +5791,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B78" s="5">
         <v>46258.6037837037</v>
@@ -5798,7 +5801,7 @@
         <v>46258.66085922453</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
@@ -5825,13 +5828,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Q78" s="5">
         <v>46426</v>
@@ -5851,7 +5854,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B79" s="9">
         <v>46258.60378907407</v>
@@ -5861,7 +5864,7 @@
         <v>46258.66118105324</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
@@ -5888,13 +5891,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q79" s="10"/>
       <c r="R79" s="10"/>
@@ -5904,7 +5907,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B80" s="5">
         <v>46258.60379219908</v>
@@ -5914,7 +5917,7 @@
         <v>46258.661176724534</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -5941,13 +5944,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -5957,7 +5960,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B81" s="9">
         <v>46258.603860243056</v>
@@ -5967,7 +5970,7 @@
         <v>46258.66085556713</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
@@ -5994,10 +5997,10 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>26</v>
@@ -6020,7 +6023,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B82" s="5">
         <v>46258.603864756944</v>
@@ -6030,7 +6033,7 @@
         <v>46258.661245509255</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6057,13 +6060,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6073,7 +6076,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B83" s="9">
         <v>46258.60386903935</v>
@@ -6083,7 +6086,7 @@
         <v>46258.66124155093</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
@@ -6110,13 +6113,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q83" s="10"/>
       <c r="R83" s="10"/>
@@ -6126,7 +6129,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B84" s="5">
         <v>46258.60390300926</v>
@@ -6136,7 +6139,7 @@
         <v>46258.660850844906</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6163,13 +6166,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Q84" s="5">
         <v>46434</v>
@@ -6189,7 +6192,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B85" s="9">
         <v>46258.60391053241</v>
@@ -6199,7 +6202,7 @@
         <v>46258.66130690972</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
@@ -6226,13 +6229,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q85" s="10"/>
       <c r="R85" s="10"/>
@@ -6242,7 +6245,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B86" s="5">
         <v>46258.60391366898</v>
@@ -6252,7 +6255,7 @@
         <v>46258.661302939814</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6279,13 +6282,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q86" s="6"/>
       <c r="R86" s="6"/>
@@ -6295,7 +6298,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B87" s="9">
         <v>46258.60393953703</v>
@@ -6305,7 +6308,7 @@
         <v>46258.65155918981</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>25</v>
@@ -6329,7 +6332,7 @@
         <v>26</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="P87" s="10" t="s">
         <v>26</v>
@@ -6342,7 +6345,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B88" s="5">
         <v>46258.603942685186</v>
@@ -6352,16 +6355,16 @@
         <v>46258.66144361111</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I88" s="5">
         <v>46435</v>
@@ -6379,13 +6382,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q88" s="5">
         <v>46436</v>
@@ -6405,7 +6408,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B89" s="9">
         <v>46258.603947407406</v>
@@ -6415,16 +6418,16 @@
         <v>46258.66140633102</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I89" s="9">
         <v>46435</v>
@@ -6442,13 +6445,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q89" s="10"/>
       <c r="R89" s="10"/>
@@ -6458,7 +6461,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B90" s="5">
         <v>46258.60395099537</v>
@@ -6468,16 +6471,16 @@
         <v>46258.66140236111</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I90" s="5">
         <v>46435</v>
@@ -6495,13 +6498,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6511,7 +6514,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B91" s="9">
         <v>46258.603988738425</v>
@@ -6521,7 +6524,7 @@
         <v>46258.66154905093</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
@@ -6548,10 +6551,10 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P91" s="10" t="s">
         <v>26</v>
@@ -6574,7 +6577,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B92" s="5">
         <v>46258.60399315972</v>
@@ -6584,7 +6587,7 @@
         <v>46258.66151215278</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -6611,13 +6614,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -6627,7 +6630,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B93" s="9">
         <v>46258.60399700231</v>
@@ -6637,7 +6640,7 @@
         <v>46258.661508379635</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -6664,13 +6667,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -6680,7 +6683,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B94" s="5">
         <v>46258.60407465277</v>
@@ -6690,16 +6693,16 @@
         <v>46258.66167725694</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I94" s="5">
         <v>46441</v>
@@ -6717,13 +6720,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q94" s="5">
         <v>46442</v>
@@ -6743,7 +6746,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B95" s="9">
         <v>46258.6040793287</v>
@@ -6753,16 +6756,16 @@
         <v>46258.661640543985</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I95" s="9">
         <v>46441</v>
@@ -6780,13 +6783,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q95" s="10"/>
       <c r="R95" s="10"/>
@@ -6796,7 +6799,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B96" s="5">
         <v>46258.60408256944</v>
@@ -6806,16 +6809,16 @@
         <v>46258.66163670139</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I96" s="5">
         <v>46441</v>
@@ -6833,13 +6836,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -6849,7 +6852,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B97" s="9">
         <v>46258.60411572916</v>
@@ -6859,16 +6862,16 @@
         <v>46258.66179225694</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I97" s="9">
         <v>46443</v>
@@ -6886,13 +6889,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q97" s="9">
         <v>46444</v>
@@ -6912,7 +6915,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B98" s="5">
         <v>46258.60412081018</v>
@@ -6922,16 +6925,16 @@
         <v>46258.66174814815</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I98" s="5">
         <v>46443</v>
@@ -6949,13 +6952,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -6965,7 +6968,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B99" s="9">
         <v>46258.60412388889</v>
@@ -6975,16 +6978,16 @@
         <v>46258.66174368055</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I99" s="9">
         <v>46443</v>
@@ -7002,13 +7005,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q99" s="10"/>
       <c r="R99" s="10"/>
@@ -7018,7 +7021,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B100" s="5">
         <v>46258.60414826389</v>
@@ -7028,7 +7031,7 @@
         <v>46258.65234785879</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>25</v>
@@ -7052,7 +7055,7 @@
         <v>26</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="P100" s="6" t="s">
         <v>26</v>
@@ -7065,7 +7068,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B101" s="9">
         <v>46258.604150694446</v>
@@ -7075,16 +7078,16 @@
         <v>46258.661866759256</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H101" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I101" s="9">
         <v>46447</v>
@@ -7102,13 +7105,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Q101" s="9">
         <v>46455</v>
@@ -7128,7 +7131,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B102" s="5">
         <v>46258.60415625</v>
@@ -7138,16 +7141,16 @@
         <v>46258.661863125</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I102" s="5">
         <v>46447</v>
@@ -7165,13 +7168,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Q102" s="5">
         <v>46455</v>

</xml_diff>